<commit_message>
Deploy current validation app
</commit_message>
<xml_diff>
--- a/Books_sellers.xlsx
+++ b/Books_sellers.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="24000" windowHeight="9480"/>
+    <workbookView windowWidth="28800" windowHeight="11580"/>
   </bookViews>
   <sheets>
     <sheet name="KE" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
     <sheet name="Categories" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">KE!$A$1:$Y$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">KE!$A$1:$Y$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Categories!$A$1:$Z$87</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="40">
   <si>
     <t>SellerName</t>
   </si>
@@ -146,6 +146,9 @@
     <t>Kabi Collections</t>
   </si>
   <si>
+    <t>Homes Decor Trends</t>
+  </si>
+  <si>
     <t>Youth Wardrobe-COD</t>
   </si>
   <si>
@@ -160,12 +163,12 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="42" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="176" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="177" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="178" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="179" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="32">
+  <fonts count="33">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -227,6 +230,12 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
@@ -746,31 +755,28 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="178" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="12" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="179" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -779,119 +785,122 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -912,10 +921,11 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -931,7 +941,7 @@
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -1589,8 +1599,10 @@
         <v>35</v>
       </c>
     </row>
-    <row r="39" ht="14.25" spans="1:1">
-      <c r="A39" s="7"/>
+    <row r="39" ht="12.75" spans="1:1">
+      <c r="A39" s="18" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="40" ht="14.25" spans="1:1">
       <c r="A40" s="7"/>
@@ -1675,31 +1687,31 @@
     </row>
     <row r="181" ht="16.5" customHeight="1"/>
     <row r="303" ht="12.75" spans="1:1">
-      <c r="A303" s="18"/>
+      <c r="A303" s="19"/>
     </row>
     <row r="304" ht="12.75" spans="1:1">
-      <c r="A304" s="18"/>
+      <c r="A304" s="19"/>
     </row>
     <row r="305" ht="12.75" spans="1:1">
-      <c r="A305" s="18"/>
+      <c r="A305" s="19"/>
     </row>
     <row r="306" ht="12.75" spans="1:1">
-      <c r="A306" s="18"/>
+      <c r="A306" s="19"/>
     </row>
     <row r="307" ht="12.75" spans="1:1">
-      <c r="A307" s="18"/>
+      <c r="A307" s="19"/>
     </row>
     <row r="309" ht="12.75" spans="1:1">
-      <c r="A309" s="18"/>
+      <c r="A309" s="19"/>
     </row>
     <row r="310" ht="12.75" spans="1:1">
-      <c r="A310" s="18"/>
+      <c r="A310" s="19"/>
     </row>
     <row r="312" ht="12.75" spans="1:1">
-      <c r="A312" s="19"/>
+      <c r="A312" s="20"/>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:Y37" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:Y38" etc:filterBottomFollowUsedRange="0">
     <extLst/>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1737,7 +1749,7 @@
     <col min="1" max="1" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customHeight="1" spans="1:1">
+    <row r="1" customHeight="1" spans="1:2">
       <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
@@ -1806,49 +1818,49 @@
       <c r="A17" s="14"/>
       <c r="B17" s="14"/>
     </row>
-    <row r="18" customHeight="1" spans="1:1">
+    <row r="18" customHeight="1" spans="1:2">
       <c r="A18" s="14"/>
     </row>
-    <row r="19" customHeight="1" spans="1:1">
+    <row r="19" customHeight="1" spans="1:2">
       <c r="A19" s="14"/>
     </row>
-    <row r="20" customHeight="1" spans="1:1">
+    <row r="20" customHeight="1" spans="1:2">
       <c r="A20" s="14"/>
     </row>
-    <row r="21" customHeight="1" spans="1:1">
+    <row r="21" customHeight="1" spans="1:2">
       <c r="A21" s="14"/>
     </row>
-    <row r="22" customHeight="1" spans="1:1">
+    <row r="22" customHeight="1" spans="1:2">
       <c r="A22" s="14"/>
     </row>
-    <row r="23" customHeight="1" spans="1:1">
+    <row r="23" customHeight="1" spans="1:2">
       <c r="A23" s="14"/>
     </row>
-    <row r="24" customHeight="1" spans="1:1">
+    <row r="24" customHeight="1" spans="1:2">
       <c r="A24" s="14"/>
     </row>
-    <row r="25" customHeight="1" spans="1:1">
+    <row r="25" customHeight="1" spans="1:2">
       <c r="A25" s="14"/>
     </row>
-    <row r="26" customHeight="1" spans="1:1">
+    <row r="26" customHeight="1" spans="1:2">
       <c r="A26" s="14"/>
     </row>
-    <row r="27" customHeight="1" spans="1:1">
+    <row r="27" customHeight="1" spans="1:2">
       <c r="A27" s="14"/>
     </row>
-    <row r="28" customHeight="1" spans="1:1">
+    <row r="28" customHeight="1" spans="1:2">
       <c r="A28" s="14"/>
     </row>
-    <row r="29" customHeight="1" spans="1:1">
+    <row r="29" customHeight="1" spans="1:2">
       <c r="A29" s="14"/>
     </row>
-    <row r="30" customHeight="1" spans="1:1">
+    <row r="30" customHeight="1" spans="1:2">
       <c r="A30" s="14"/>
     </row>
-    <row r="31" customHeight="1" spans="1:1">
+    <row r="31" customHeight="1" spans="1:2">
       <c r="A31" s="14"/>
     </row>
-    <row r="32" customHeight="1" spans="1:1">
+    <row r="32" customHeight="1" spans="1:2">
       <c r="A32" s="14"/>
     </row>
     <row r="33" customHeight="1" spans="1:1">
@@ -13484,58 +13496,58 @@
     <row r="48" customHeight="1" spans="1:1">
       <c r="A48" s="3"/>
     </row>
-    <row r="49" customHeight="1" spans="1:1">
+    <row r="49" customHeight="1" spans="1:2">
       <c r="A49" s="3"/>
     </row>
-    <row r="50" customHeight="1" spans="1:1">
+    <row r="50" customHeight="1" spans="1:2">
       <c r="A50" s="3"/>
     </row>
-    <row r="51" customHeight="1" spans="1:1">
+    <row r="51" customHeight="1" spans="1:2">
       <c r="A51" s="3"/>
     </row>
-    <row r="52" customHeight="1" spans="1:1">
+    <row r="52" customHeight="1" spans="1:2">
       <c r="A52" s="3"/>
     </row>
-    <row r="53" customHeight="1" spans="1:1">
+    <row r="53" customHeight="1" spans="1:2">
       <c r="A53" s="3"/>
     </row>
-    <row r="54" customHeight="1" spans="1:1">
+    <row r="54" customHeight="1" spans="1:2">
       <c r="A54" s="3"/>
     </row>
-    <row r="55" customHeight="1" spans="1:1">
+    <row r="55" customHeight="1" spans="1:2">
       <c r="A55" s="3"/>
     </row>
-    <row r="56" customHeight="1" spans="1:1">
+    <row r="56" customHeight="1" spans="1:2">
       <c r="A56" s="3"/>
     </row>
-    <row r="57" customHeight="1" spans="1:1">
+    <row r="57" customHeight="1" spans="1:2">
       <c r="A57" s="3"/>
     </row>
-    <row r="58" customHeight="1" spans="1:1">
+    <row r="58" customHeight="1" spans="1:2">
       <c r="A58" s="3"/>
     </row>
-    <row r="59" customHeight="1" spans="1:1">
+    <row r="59" customHeight="1" spans="1:2">
       <c r="A59" s="3"/>
     </row>
-    <row r="60" customHeight="1" spans="1:1">
+    <row r="60" customHeight="1" spans="1:2">
       <c r="A60" s="3"/>
     </row>
     <row r="61" customHeight="1" spans="1:2">
       <c r="A61" s="3"/>
       <c r="B61" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="62" customHeight="1" spans="1:2">
       <c r="A62" s="3"/>
       <c r="B62" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
-    <row r="63" customHeight="1" spans="1:1">
+    <row r="63" customHeight="1" spans="1:2">
       <c r="A63" s="3"/>
     </row>
-    <row r="64" customHeight="1" spans="1:1">
+    <row r="64" customHeight="1" spans="1:2">
       <c r="A64" s="3"/>
     </row>
     <row r="65" customHeight="1" spans="1:1">
@@ -18357,7 +18369,7 @@
   <sheetData>
     <row r="1" customHeight="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" customHeight="1" spans="1:1">

</xml_diff>